<commit_message>
feat(project-detail): update template to better guide usesr
</commit_message>
<xml_diff>
--- a/frontend/public/metadata_template.xlsx
+++ b/frontend/public/metadata_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cells" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cells" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -143,7 +143,8 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Required. Must equal the number in each cell's cycling filename.</t>
+        <t>The cycling data file you upload must contain this ID No in its filename.
+Examples: 12_cycling.xlsx / CEL-12_data.csv</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -746,7 +747,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: document custom metadata columns and show them in the template
Explain in the metadata guide that any extra column is kept with the cell,
displayed on the cell card, and offered as a hierarchy level when it can group
cells (2+ distinct values) — identical for uploads and DIGIBAT. Add example
extra columns to the metadata template to demonstrate.
</commit_message>
<xml_diff>
--- a/frontend/public/metadata_template.xlsx
+++ b/frontend/public/metadata_template.xlsx
@@ -143,8 +143,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>The cycling data file you upload must contain this ID No in its filename.
-Examples: 12_cycling.xlsx / CEL-12_data.csv</t>
+        <t>Required. Must equal the number in each cell's cycling filename.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -155,6 +154,11 @@
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Matched by value, so 1 and 1.0 are the same condition.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Columns beyond the standard set are preserved as-is, shown on the cell card, and selectable as a hierarchy filter — add any you need.</t>
       </text>
     </comment>
   </commentList>
@@ -450,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -474,6 +478,9 @@
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
     <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -582,6 +589,21 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Cathode supplier</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Electrolyte supplier</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Testing procedure</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -667,6 +689,21 @@
           <t>first replicate</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Canrud</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Canrud</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>rate performance</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -745,6 +782,22 @@
       <c r="T3" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Canrud</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Canrud</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>formation</t>
         </is>
       </c>
     </row>

</xml_diff>